<commit_message>
Work in progress: FG payment reconciliation, quote policy period, web date input
tf-api:
- FG payment recon points at the bare .asmx SOAP endpoint from the live WSDL;
  the transport now picks SOAP vs form-urlencoded encoding per URL form
- quotes gain policyStartDate/policyEndDate (migration 20260806095258)
- FG provider, mapper, normalizer and http updates with test coverage

tf-web:
- new DateInput component (dd/mm/yyyy presentation, ISO internally) + tests
- addon-selection module extracted with tests; quote-request tests added
- compare, proposal, vehicle-details and new-vehicle pages updated

Committed as-is to clear the tree before the HDFC ERGO provider work.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tf-api/docs/Private Car- Web Aggregator.xlsx
+++ b/tf-api/docs/Private Car- Web Aggregator.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30228"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B5E9269-AD2E-4897-9C49-0EA434C3D0AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet sheetId="1" name="Testcases" state="visible" r:id="rId4"/>
-    <sheet sheetId="4" name="Screenshots" state="visible" r:id="rId5"/>
-    <sheet sheetId="3" name="Partner Frontend validation" state="hidden" r:id="rId6"/>
+    <sheet name="Testcases" sheetId="1" r:id="rId1"/>
+    <sheet name="Screen shots" sheetId="5" r:id="rId2"/>
+    <sheet name="Partner Frontend validation" sheetId="3" state="hidden" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase">Testcases!$A$1:$L$38</definedName>
@@ -19,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="431" uniqueCount="292">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="445" uniqueCount="267">
   <si>
     <t>Sr. No</t>
   </si>
@@ -327,7 +328,7 @@
     <t>In case of Rollover case PUC is mandatory. Two fields should be added as PUC No, and PUC Expiry Date</t>
   </si>
   <si>
-    <t xml:space="preserve">If we have selected Valid PUC flag "YES" then following field should be Mandatory.
+    <t>If we have selected Valid PUC flag "YES" then following field should be Mandatory.
 1. PUC No
 2. PUC Expiry Date</t>
   </si>
@@ -380,7 +381,7 @@
     <t>Inspection wavier for Third Party Policy</t>
   </si>
   <si>
-    <t xml:space="preserve">Policy period (Risk Start Date) should be taken after T+2 days ( i.e. 1. Payment collected date is 09/05/2024 then Risk start date should be 12/05/2024.  
+    <t>Policy period (Risk Start Date) should be taken after T+2 days ( i.e. 1. Payment collected date is 09/05/2024 then Risk start date should be 12/05/2024.  
 2. Issuance time should be pass at the time of policy issuance. Payment collected date is 09/05/2024 04:00:00 then Risk start date should be 11/05/2024 04:01:00.)</t>
   </si>
   <si>
@@ -576,7 +577,7 @@
     <t>Decline RTO code - Haryana</t>
   </si>
   <si>
-    <t xml:space="preserve">System should not be allowed to issued policy with Decline RTO code.
+    <t>System should not be allowed to issued policy with Decline RTO code.
 HR-38</t>
   </si>
   <si>
@@ -763,88 +764,10 @@
     <t>CKYC Verification fail &amp; document uploading</t>
   </si>
   <si>
-    <t xml:space="preserve">CKYC Verification failed if Wrong PAN or DOB details updated. </t>
+    <t>CKYC Verification failed if Wrong PAN or DOB details updated. </t>
   </si>
   <si>
     <t>[tf-api FG] CKYC verification with WRONG PAN (ABCDE1234F) correctly FAILS (no CKYC record) — portal offers Aadhaar and OVD document-upload fallbacks. Valid PAN DHQPG4064J → CKYC 40053862382888 (Meenu Gupta). (Identity scenario — no vehicle participates.)</t>
-  </si>
-  <si>
-    <t>tf-api FG provider — customer journey screen by screen (live portal http://localhost:8080 → tf-api → live FG UAT). Each screen lists the test cases it evidences.</t>
-  </si>
-  <si>
-    <t>Screen 1 — Home / product selection</t>
-  </si>
-  <si>
-    <t>Applies to: All journeys (TC_01–TC_05, TC_24, TC_25)</t>
-  </si>
-  <si>
-    <t>Screen 2 — Login (registered mobile)</t>
-  </si>
-  <si>
-    <t>Applies to: All journeys</t>
-  </si>
-  <si>
-    <t>Screen 3 — Car number entry (DL10CN1591)</t>
-  </si>
-  <si>
-    <t>Applies to: TC_03, TC_07, TC_21, TC_25, TC_30</t>
-  </si>
-  <si>
-    <t>Screen 4 — RC details auto-fetched (Honda City, prev insurer + expiry)</t>
-  </si>
-  <si>
-    <t>Applies to: TC_03, TC_07, TC_25, TC_30</t>
-  </si>
-  <si>
-    <t>Screen 5 — Plans (Comprehensive): live compare, IDV control, NCB, claim toggle</t>
-  </si>
-  <si>
-    <t>Applies to: TC_03, TC_07 (IDV band), TC_25</t>
-  </si>
-  <si>
-    <t>Screen 6 — Plans (Third-Party): FG not offered (GCI UW block) — ICICI only</t>
-  </si>
-  <si>
-    <t>Applies to: TC_04</t>
-  </si>
-  <si>
-    <t>Screen 7 — Plans (Standalone OD): previous TP policy details required</t>
-  </si>
-  <si>
-    <t>Applies to: TC_02, TC_13, TC_14</t>
-  </si>
-  <si>
-    <t>Screen 8 — Plans with NCB 25% selected (premium reprices)</t>
-  </si>
-  <si>
-    <t>Applies to: TC_13, TC_21</t>
-  </si>
-  <si>
-    <t>Screen 9 — FG 45-day advance-inception message on the compare card</t>
-  </si>
-  <si>
-    <t>Applies to: TC_30</t>
-  </si>
-  <si>
-    <t>Screen 10 — New car (no reg yet): manual make/model + RTO + purchase date</t>
-  </si>
-  <si>
-    <t>Applies to: TC_01, TC_05, TC_24 (F13 journey)</t>
-  </si>
-  <si>
-    <t>Screen 11 — Proposer details (DOB/gender/address, engine &amp; chassis, nominee/CPA)</t>
-  </si>
-  <si>
-    <t>Applies to: TC_01–TC_03, TC_06</t>
-  </si>
-  <si>
-    <t>Screen 12 — KYC FAILS for wrong PAN → Aadhaar / OVD document-upload fallback</t>
-  </si>
-  <si>
-    <t>Applies to: TC_37</t>
-  </si>
-  <si>
-    <t>Note: FG-priced UI screens (FG premium card / add-on panel / review breakdown) pend FG UAT stability; the equivalent API evidence (11+ real policy numbers) is in the Testcases sheet.</t>
   </si>
   <si>
     <t>Note : These are the Buisness core validation. TCS service will throw these error message that need to be shown/ display on portal frontend.</t>
@@ -901,71 +824,54 @@
   </si>
   <si>
     <t>Pop up message should  display , Same Registration Number exists in Active.</t>
+  </si>
+  <si>
+    <t>ScreenSHots</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="11" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
     <font>
       <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
       <sz val="11"/>
       <name val="Calibri"/>
-    </font>
-    <font>
-      <b/>
-    </font>
-    <font>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
     <font>
       <sz val="11"/>
       <name val="Montserrat"/>
     </font>
     <font>
+      <sz val="10"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="10"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="12"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <i/>
-      <color rgb="FF555555"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="10"/>
     </font>
     <font>
       <b/>
       <u/>
+      <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="6">
@@ -977,7 +883,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.7999816888943144"/>
+        <fgColor theme="5" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -989,7 +895,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.3999755851924192"/>
+        <fgColor theme="7" tint="0.39997558519241921"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1027,7 +933,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -1035,55 +941,37 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1101,479 +989,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:oneCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>4</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="6858000" cy="3810000"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="Picture 1">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="0"/>
-          <a:ext cx="0" cy="0"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>28</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="6858000" cy="3810000"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Picture 2">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2" cstate="print"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="0"/>
-          <a:ext cx="0" cy="0"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>52</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="6858000" cy="3810000"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="Picture 3">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3" cstate="print"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="0"/>
-          <a:ext cx="0" cy="0"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>76</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="6858000" cy="3810000"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="4" name="Picture 4">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4" cstate="print"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="0"/>
-          <a:ext cx="0" cy="0"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>100</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="6858000" cy="3810000"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="5" name="Picture 5">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId5" cstate="print"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="0"/>
-          <a:ext cx="0" cy="0"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>124</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="6858000" cy="3810000"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="6" name="Picture 6">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId6" cstate="print"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="0"/>
-          <a:ext cx="0" cy="0"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>148</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="6858000" cy="3810000"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="7" name="Picture 7">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId7" cstate="print"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="0"/>
-          <a:ext cx="0" cy="0"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>172</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="6858000" cy="3810000"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="8" name="Picture 8">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId8" cstate="print"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="0"/>
-          <a:ext cx="0" cy="0"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>196</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="6858000" cy="3810000"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="9" name="Picture 9">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId9" cstate="print"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="0"/>
-          <a:ext cx="0" cy="0"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>220</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="6858000" cy="3810000"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="10" name="Picture 10">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId10" cstate="print"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="0"/>
-          <a:ext cx="0" cy="0"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>244</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="6858000" cy="3810000"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="11" name="Picture 11">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId11" cstate="print"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="0"/>
-          <a:ext cx="0" cy="0"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>268</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="6858000" cy="3810000"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="12" name="Picture 12">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId12" cstate="print"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="0"/>
-          <a:ext cx="0" cy="0"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:oneCellAnchor>
-</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1838,29 +1253,30 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <tabColor rgb="FFFF0000"/>
   </sheetPr>
   <dimension ref="A1:L38"/>
-  <sheetFormatPr defaultRowHeight="14.45" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="25" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="25" defaultRowHeight="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="3.5703125" style="1" customWidth="1"/>
-    <col min="2" max="2" width="7.42578125" style="1" customWidth="1"/>
-    <col min="3" max="3" width="7.7109375" style="1" customWidth="1"/>
-    <col min="4" max="4" width="8.5703125" style="1" customWidth="1"/>
-    <col min="5" max="5" width="24.7109375" style="1" customWidth="1"/>
-    <col min="6" max="6" width="38.28515625" style="1" customWidth="1"/>
-    <col min="7" max="7" width="37.5703125" style="1" customWidth="1"/>
-    <col min="8" max="8" width="12.5703125" style="1" customWidth="1"/>
-    <col min="9" max="9" width="27.5703125" style="1" customWidth="1"/>
-    <col min="10" max="10" width="11.7109375" style="1" customWidth="1"/>
+    <col min="1" max="1" width="3.5546875" style="1" customWidth="1"/>
+    <col min="2" max="2" width="7.44140625" style="1" customWidth="1"/>
+    <col min="3" max="3" width="7.6640625" style="1" customWidth="1"/>
+    <col min="4" max="4" width="8.5546875" style="1" customWidth="1"/>
+    <col min="5" max="5" width="24.6640625" style="1" customWidth="1"/>
+    <col min="6" max="6" width="38.33203125" style="1" customWidth="1"/>
+    <col min="7" max="7" width="37.5546875" style="1" customWidth="1"/>
+    <col min="8" max="8" width="12.5546875" style="1" customWidth="1"/>
+    <col min="9" max="9" width="27.5546875" style="1" customWidth="1"/>
+    <col min="10" max="10" width="11.6640625" style="1" customWidth="1"/>
     <col min="11" max="11" width="26" style="1" customWidth="1"/>
     <col min="12" max="12" width="34" style="1" customWidth="1"/>
-    <col min="13" max="16384" width="25" style="1" customWidth="1"/>
+    <col min="13" max="13" width="25" style="1" customWidth="1"/>
+    <col min="14" max="16384" width="25" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="28.9" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12" ht="28.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -1891,42 +1307,42 @@
       <c r="J1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="3" t="s">
+      <c r="K1" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="3" t="s">
+      <c r="L1" s="2" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="2" ht="28.9" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A2" s="4">
+    <row r="2" spans="1:12" ht="28.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="3">
         <v>1</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="B2" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="C2" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="D2" s="4" t="s">
+      <c r="C2" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="D2" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="E2" s="4" t="s">
+      <c r="E2" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="F2" s="4" t="s">
+      <c r="F2" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="G2" s="4" t="s">
+      <c r="G2" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="H2" s="4" t="s">
+      <c r="H2" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="I2" s="4" t="s">
+      <c r="I2" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="J2" s="4">
+      <c r="J2" s="3">
         <v>1</v>
       </c>
       <c r="K2" s="1" t="s">
@@ -1936,35 +1352,35 @@
         <v>21</v>
       </c>
     </row>
-    <row r="3" ht="28.9" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A3" s="4">
+    <row r="3" spans="1:12" ht="28.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="3">
         <v>2</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="B3" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="C3" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="D3" s="4" t="s">
+      <c r="C3" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="D3" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="E3" s="4" t="s">
+      <c r="E3" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="F3" s="4" t="s">
+      <c r="F3" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="G3" s="4" t="s">
+      <c r="G3" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="H3" s="4" t="s">
+      <c r="H3" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="I3" s="4" t="s">
+      <c r="I3" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="J3" s="4">
+      <c r="J3" s="3">
         <v>2</v>
       </c>
       <c r="K3" s="1" t="s">
@@ -1974,35 +1390,35 @@
         <v>27</v>
       </c>
     </row>
-    <row r="4" ht="28.9" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A4" s="4">
+    <row r="4" spans="1:12" ht="28.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="3">
         <v>3</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="B4" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="C4" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="D4" s="4" t="s">
+      <c r="C4" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="D4" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="E4" s="4" t="s">
+      <c r="E4" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="F4" s="4" t="s">
+      <c r="F4" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="G4" s="4" t="s">
+      <c r="G4" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="H4" s="4" t="s">
+      <c r="H4" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="I4" s="4" t="s">
+      <c r="I4" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="J4" s="4">
+      <c r="J4" s="3">
         <v>3</v>
       </c>
       <c r="K4" s="1" t="s">
@@ -2012,35 +1428,35 @@
         <v>27</v>
       </c>
     </row>
-    <row r="5" ht="28.9" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A5" s="4">
+    <row r="5" spans="1:12" ht="28.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="3">
         <v>4</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="B5" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="C5" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="D5" s="4" t="s">
+      <c r="C5" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="D5" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="E5" s="4" t="s">
+      <c r="E5" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="F5" s="4" t="s">
+      <c r="F5" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="G5" s="4" t="s">
+      <c r="G5" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="H5" s="4" t="s">
+      <c r="H5" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="I5" s="4" t="s">
+      <c r="I5" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="J5" s="4">
+      <c r="J5" s="3">
         <v>4</v>
       </c>
       <c r="K5" s="1" t="s">
@@ -2050,73 +1466,73 @@
         <v>37</v>
       </c>
     </row>
-    <row r="6" ht="28.9" customHeight="1" spans="1:12" s="5" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="4">
+    <row r="6" spans="1:12" s="4" customFormat="1" ht="28.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="3">
         <v>5</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="B6" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="C6" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="D6" s="4" t="s">
+      <c r="C6" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="D6" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="E6" s="4" t="s">
+      <c r="E6" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="F6" s="4" t="s">
+      <c r="F6" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="G6" s="4" t="s">
+      <c r="G6" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="H6" s="4" t="s">
+      <c r="H6" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="I6" s="4" t="s">
+      <c r="I6" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="J6" s="4">
+      <c r="J6" s="3">
         <v>5</v>
       </c>
-      <c r="K6" s="5" t="s">
+      <c r="K6" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="L6" s="5" t="s">
+      <c r="L6" s="4" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="7" ht="115.15" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A7" s="4">
+    <row r="7" spans="1:12" ht="115.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="3">
         <v>6</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="B7" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="C7" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="D7" s="4" t="s">
+      <c r="C7" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="D7" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="E7" s="4" t="s">
+      <c r="E7" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="F7" s="4" t="s">
+      <c r="F7" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="G7" s="4" t="s">
+      <c r="G7" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="H7" s="4" t="s">
+      <c r="H7" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="I7" s="6" t="s">
+      <c r="I7" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="J7" s="4">
+      <c r="J7" s="3">
         <v>6</v>
       </c>
       <c r="K7" s="1" t="s">
@@ -2126,35 +1542,35 @@
         <v>51</v>
       </c>
     </row>
-    <row r="8" ht="100.9" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A8" s="4">
+    <row r="8" spans="1:12" ht="100.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="3">
         <v>7</v>
       </c>
-      <c r="B8" s="4" t="s">
+      <c r="B8" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="C8" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="D8" s="4" t="s">
+      <c r="C8" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="D8" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="E8" s="4" t="s">
+      <c r="E8" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="F8" s="4" t="s">
+      <c r="F8" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="G8" s="4" t="s">
+      <c r="G8" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="H8" s="4" t="s">
+      <c r="H8" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="I8" s="4" t="s">
+      <c r="I8" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="J8" s="4">
+      <c r="J8" s="3">
         <v>7</v>
       </c>
       <c r="K8" s="1" t="s">
@@ -2164,35 +1580,35 @@
         <v>59</v>
       </c>
     </row>
-    <row r="9" ht="115.15" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A9" s="4">
+    <row r="9" spans="1:12" ht="115.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="3">
         <v>8</v>
       </c>
-      <c r="B9" s="4" t="s">
+      <c r="B9" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="C9" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="D9" s="4" t="s">
+      <c r="C9" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="D9" s="3" t="s">
         <v>61</v>
       </c>
-      <c r="E9" s="4" t="s">
+      <c r="E9" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="F9" s="4" t="s">
+      <c r="F9" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="G9" s="4" t="s">
+      <c r="G9" s="3" t="s">
         <v>64</v>
       </c>
-      <c r="H9" s="4" t="s">
+      <c r="H9" s="3" t="s">
         <v>65</v>
       </c>
-      <c r="I9" s="4" t="s">
+      <c r="I9" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="J9" s="4">
+      <c r="J9" s="3">
         <v>8</v>
       </c>
       <c r="K9" s="1" t="s">
@@ -2202,35 +1618,35 @@
         <v>37</v>
       </c>
     </row>
-    <row r="10" ht="144" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A10" s="4">
+    <row r="10" spans="1:12" ht="144" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="3">
         <v>9</v>
       </c>
-      <c r="B10" s="4" t="s">
+      <c r="B10" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="C10" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="D10" s="4" t="s">
+      <c r="C10" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="D10" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="E10" s="7" t="s">
+      <c r="E10" s="6" t="s">
         <v>70</v>
       </c>
-      <c r="F10" s="7" t="s">
+      <c r="F10" s="6" t="s">
         <v>71</v>
       </c>
-      <c r="G10" s="4" t="s">
+      <c r="G10" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="H10" s="4" t="s">
+      <c r="H10" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="I10" s="4" t="s">
+      <c r="I10" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="J10" s="4">
+      <c r="J10" s="3">
         <v>9</v>
       </c>
       <c r="K10" s="1" t="s">
@@ -2240,35 +1656,35 @@
         <v>37</v>
       </c>
     </row>
-    <row r="11" ht="43.15" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A11" s="4">
+    <row r="11" spans="1:12" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="3">
         <v>10</v>
       </c>
-      <c r="B11" s="4" t="s">
+      <c r="B11" s="3" t="s">
         <v>75</v>
       </c>
-      <c r="C11" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="D11" s="4" t="s">
+      <c r="C11" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="D11" s="3" t="s">
         <v>76</v>
       </c>
-      <c r="E11" s="4" t="s">
+      <c r="E11" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="F11" s="4" t="s">
+      <c r="F11" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="G11" s="4" t="s">
+      <c r="G11" s="3" t="s">
         <v>79</v>
       </c>
-      <c r="H11" s="4" t="s">
+      <c r="H11" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="I11" s="4" t="s">
+      <c r="I11" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="J11" s="4">
+      <c r="J11" s="3">
         <v>10</v>
       </c>
       <c r="K11" s="1" t="s">
@@ -2278,35 +1694,35 @@
         <v>82</v>
       </c>
     </row>
-    <row r="12" ht="43.15" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A12" s="4">
+    <row r="12" spans="1:12" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="3">
         <v>11</v>
       </c>
-      <c r="B12" s="4" t="s">
+      <c r="B12" s="3" t="s">
         <v>83</v>
       </c>
-      <c r="C12" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="D12" s="4" t="s">
+      <c r="C12" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="D12" s="3" t="s">
         <v>76</v>
       </c>
-      <c r="E12" s="4" t="s">
+      <c r="E12" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="F12" s="4" t="s">
+      <c r="F12" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="G12" s="4" t="s">
+      <c r="G12" s="3" t="s">
         <v>79</v>
       </c>
-      <c r="H12" s="4" t="s">
+      <c r="H12" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="I12" s="4" t="s">
+      <c r="I12" s="3" t="s">
         <v>85</v>
       </c>
-      <c r="J12" s="4">
+      <c r="J12" s="3">
         <v>11</v>
       </c>
       <c r="K12" s="1" t="s">
@@ -2316,35 +1732,35 @@
         <v>87</v>
       </c>
     </row>
-    <row r="13" ht="43.15" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A13" s="4">
+    <row r="13" spans="1:12" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="3">
         <v>12</v>
       </c>
-      <c r="B13" s="4" t="s">
+      <c r="B13" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="C13" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="D13" s="4" t="s">
+      <c r="C13" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="D13" s="3" t="s">
         <v>76</v>
       </c>
-      <c r="E13" s="4" t="s">
+      <c r="E13" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="F13" s="4" t="s">
+      <c r="F13" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="G13" s="4" t="s">
+      <c r="G13" s="3" t="s">
         <v>79</v>
       </c>
-      <c r="H13" s="4" t="s">
+      <c r="H13" s="3" t="s">
         <v>65</v>
       </c>
-      <c r="I13" s="4" t="s">
+      <c r="I13" s="3" t="s">
         <v>90</v>
       </c>
-      <c r="J13" s="4">
+      <c r="J13" s="3">
         <v>12</v>
       </c>
       <c r="K13" s="1" t="s">
@@ -2354,35 +1770,35 @@
         <v>37</v>
       </c>
     </row>
-    <row r="14" ht="43.15" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A14" s="4">
-        <v>13</v>
-      </c>
-      <c r="B14" s="4" t="s">
+    <row r="14" spans="1:12" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="3">
+        <v>13</v>
+      </c>
+      <c r="B14" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="C14" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="D14" s="4" t="s">
+      <c r="C14" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="D14" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="E14" s="4" t="s">
+      <c r="E14" s="3" t="s">
         <v>94</v>
       </c>
-      <c r="F14" s="4" t="s">
+      <c r="F14" s="3" t="s">
         <v>95</v>
       </c>
-      <c r="G14" s="4" t="s">
+      <c r="G14" s="3" t="s">
         <v>95</v>
       </c>
-      <c r="H14" s="4" t="s">
+      <c r="H14" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="I14" s="4" t="s">
+      <c r="I14" s="3" t="s">
         <v>96</v>
       </c>
-      <c r="J14" s="4">
+      <c r="J14" s="3">
         <v>13</v>
       </c>
       <c r="K14" s="1" t="s">
@@ -2392,35 +1808,35 @@
         <v>27</v>
       </c>
     </row>
-    <row r="15" ht="57.6" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A15" s="4">
+    <row r="15" spans="1:12" ht="57.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="3">
         <v>14</v>
       </c>
-      <c r="B15" s="4" t="s">
+      <c r="B15" s="3" t="s">
         <v>98</v>
       </c>
-      <c r="C15" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="D15" s="4" t="s">
+      <c r="C15" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="D15" s="3" t="s">
         <v>99</v>
       </c>
-      <c r="E15" s="7" t="s">
+      <c r="E15" s="6" t="s">
         <v>100</v>
       </c>
-      <c r="F15" s="7" t="s">
+      <c r="F15" s="6" t="s">
         <v>101</v>
       </c>
-      <c r="G15" s="4" t="s">
+      <c r="G15" s="3" t="s">
         <v>102</v>
       </c>
-      <c r="H15" s="4" t="s">
+      <c r="H15" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="I15" s="4" t="s">
+      <c r="I15" s="3" t="s">
         <v>103</v>
       </c>
-      <c r="J15" s="4">
+      <c r="J15" s="3">
         <v>14</v>
       </c>
       <c r="K15" s="1" t="s">
@@ -2430,35 +1846,35 @@
         <v>37</v>
       </c>
     </row>
-    <row r="16" ht="72" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A16" s="4">
+    <row r="16" spans="1:12" ht="72" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="3">
         <v>15</v>
       </c>
-      <c r="B16" s="4" t="s">
+      <c r="B16" s="3" t="s">
         <v>105</v>
       </c>
-      <c r="C16" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="D16" s="4" t="s">
+      <c r="C16" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="D16" s="3" t="s">
         <v>106</v>
       </c>
-      <c r="E16" s="4" t="s">
+      <c r="E16" s="3" t="s">
         <v>107</v>
       </c>
-      <c r="F16" s="8" t="s">
+      <c r="F16" s="7" t="s">
         <v>108</v>
       </c>
-      <c r="G16" s="4" t="s">
+      <c r="G16" s="3" t="s">
         <v>109</v>
       </c>
-      <c r="H16" s="4" t="s">
+      <c r="H16" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="I16" s="9" t="s">
+      <c r="I16" s="8" t="s">
         <v>110</v>
       </c>
-      <c r="J16" s="4">
+      <c r="J16" s="3">
         <v>15</v>
       </c>
       <c r="K16" s="1" t="s">
@@ -2468,35 +1884,35 @@
         <v>37</v>
       </c>
     </row>
-    <row r="17" ht="72" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A17" s="4">
+    <row r="17" spans="1:12" ht="72" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="3">
         <v>16</v>
       </c>
-      <c r="B17" s="4" t="s">
+      <c r="B17" s="3" t="s">
         <v>112</v>
       </c>
-      <c r="C17" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="D17" s="4" t="s">
+      <c r="C17" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="D17" s="3" t="s">
         <v>106</v>
       </c>
-      <c r="E17" s="4" t="s">
+      <c r="E17" s="3" t="s">
         <v>113</v>
       </c>
-      <c r="F17" s="8" t="s">
+      <c r="F17" s="7" t="s">
         <v>108</v>
       </c>
-      <c r="G17" s="4" t="s">
+      <c r="G17" s="3" t="s">
         <v>109</v>
       </c>
-      <c r="H17" s="4" t="s">
+      <c r="H17" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="I17" s="9" t="s">
+      <c r="I17" s="8" t="s">
         <v>114</v>
       </c>
-      <c r="J17" s="4">
+      <c r="J17" s="3">
         <v>16</v>
       </c>
       <c r="K17" s="1" t="s">
@@ -2506,35 +1922,35 @@
         <v>27</v>
       </c>
     </row>
-    <row r="18" ht="137.25" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A18" s="4">
+    <row r="18" spans="1:12" ht="137.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="3">
         <v>17</v>
       </c>
-      <c r="B18" s="4" t="s">
+      <c r="B18" s="3" t="s">
         <v>116</v>
       </c>
-      <c r="C18" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="D18" s="4" t="s">
+      <c r="C18" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="D18" s="3" t="s">
         <v>106</v>
       </c>
-      <c r="E18" s="7" t="s">
+      <c r="E18" s="6" t="s">
         <v>117</v>
       </c>
-      <c r="F18" s="8" t="s">
+      <c r="F18" s="7" t="s">
         <v>118</v>
       </c>
-      <c r="G18" s="7" t="s">
+      <c r="G18" s="6" t="s">
         <v>119</v>
       </c>
-      <c r="H18" s="4" t="s">
+      <c r="H18" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="I18" s="4" t="s">
+      <c r="I18" s="3" t="s">
         <v>120</v>
       </c>
-      <c r="J18" s="4">
+      <c r="J18" s="3">
         <v>17</v>
       </c>
       <c r="K18" s="1" t="s">
@@ -2544,35 +1960,35 @@
         <v>37</v>
       </c>
     </row>
-    <row r="19" ht="165.6" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A19" s="4">
+    <row r="19" spans="1:12" ht="165.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="3">
         <v>18</v>
       </c>
-      <c r="B19" s="4" t="s">
+      <c r="B19" s="3" t="s">
         <v>122</v>
       </c>
-      <c r="C19" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="D19" s="4" t="s">
+      <c r="C19" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="D19" s="3" t="s">
         <v>106</v>
       </c>
-      <c r="E19" s="4" t="s">
+      <c r="E19" s="3" t="s">
         <v>107</v>
       </c>
-      <c r="F19" s="8" t="s">
+      <c r="F19" s="7" t="s">
         <v>123</v>
       </c>
-      <c r="G19" s="10" t="s">
+      <c r="G19" s="9" t="s">
         <v>124</v>
       </c>
-      <c r="H19" s="4" t="s">
+      <c r="H19" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="I19" s="9" t="s">
+      <c r="I19" s="8" t="s">
         <v>125</v>
       </c>
-      <c r="J19" s="4">
+      <c r="J19" s="3">
         <v>18</v>
       </c>
       <c r="K19" s="1" t="s">
@@ -2582,35 +1998,35 @@
         <v>37</v>
       </c>
     </row>
-    <row r="20" ht="165.6" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A20" s="4">
+    <row r="20" spans="1:12" ht="165.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="3">
         <v>19</v>
       </c>
-      <c r="B20" s="4" t="s">
+      <c r="B20" s="3" t="s">
         <v>127</v>
       </c>
-      <c r="C20" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="D20" s="4" t="s">
+      <c r="C20" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="D20" s="3" t="s">
         <v>106</v>
       </c>
-      <c r="E20" s="4" t="s">
+      <c r="E20" s="3" t="s">
         <v>128</v>
       </c>
-      <c r="F20" s="8" t="s">
+      <c r="F20" s="7" t="s">
         <v>123</v>
       </c>
-      <c r="G20" s="10" t="s">
+      <c r="G20" s="9" t="s">
         <v>124</v>
       </c>
-      <c r="H20" s="4" t="s">
+      <c r="H20" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="I20" s="9" t="s">
+      <c r="I20" s="8" t="s">
         <v>129</v>
       </c>
-      <c r="J20" s="4">
+      <c r="J20" s="3">
         <v>19</v>
       </c>
       <c r="K20" s="1" t="s">
@@ -2620,35 +2036,35 @@
         <v>37</v>
       </c>
     </row>
-    <row r="21" ht="43.15" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A21" s="4">
+    <row r="21" spans="1:12" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A21" s="3">
         <v>20</v>
       </c>
-      <c r="B21" s="4" t="s">
+      <c r="B21" s="3" t="s">
         <v>131</v>
       </c>
-      <c r="C21" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="D21" s="4" t="s">
+      <c r="C21" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="D21" s="3" t="s">
         <v>106</v>
       </c>
-      <c r="E21" s="7" t="s">
+      <c r="E21" s="6" t="s">
         <v>132</v>
       </c>
-      <c r="F21" s="7" t="s">
+      <c r="F21" s="6" t="s">
         <v>133</v>
       </c>
-      <c r="G21" s="7" t="s">
+      <c r="G21" s="6" t="s">
         <v>134</v>
       </c>
-      <c r="H21" s="4" t="s">
+      <c r="H21" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="I21" s="4" t="s">
+      <c r="I21" s="3" t="s">
         <v>135</v>
       </c>
-      <c r="J21" s="4">
+      <c r="J21" s="3">
         <v>20</v>
       </c>
       <c r="K21" s="1" t="s">
@@ -2658,35 +2074,35 @@
         <v>37</v>
       </c>
     </row>
-    <row r="22" ht="43.15" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A22" s="4">
+    <row r="22" spans="1:12" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A22" s="3">
         <v>21</v>
       </c>
-      <c r="B22" s="4" t="s">
+      <c r="B22" s="3" t="s">
         <v>137</v>
       </c>
-      <c r="C22" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="D22" s="4" t="s">
+      <c r="C22" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="D22" s="3" t="s">
         <v>138</v>
       </c>
-      <c r="E22" s="4" t="s">
+      <c r="E22" s="3" t="s">
         <v>139</v>
       </c>
-      <c r="F22" s="4" t="s">
+      <c r="F22" s="3" t="s">
         <v>140</v>
       </c>
-      <c r="G22" s="7" t="s">
+      <c r="G22" s="6" t="s">
         <v>141</v>
       </c>
-      <c r="H22" s="4" t="s">
+      <c r="H22" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="I22" s="4" t="s">
+      <c r="I22" s="3" t="s">
         <v>142</v>
       </c>
-      <c r="J22" s="4">
+      <c r="J22" s="3">
         <v>21</v>
       </c>
       <c r="K22" s="1" t="s">
@@ -2696,35 +2112,35 @@
         <v>27</v>
       </c>
     </row>
-    <row r="23" ht="43.15" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A23" s="4">
+    <row r="23" spans="1:12" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A23" s="3">
         <v>22</v>
       </c>
-      <c r="B23" s="4" t="s">
+      <c r="B23" s="3" t="s">
         <v>144</v>
       </c>
-      <c r="C23" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="D23" s="4" t="s">
+      <c r="C23" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="D23" s="3" t="s">
         <v>145</v>
       </c>
-      <c r="E23" s="7" t="s">
+      <c r="E23" s="6" t="s">
         <v>146</v>
       </c>
-      <c r="F23" s="7" t="s">
+      <c r="F23" s="6" t="s">
         <v>147</v>
       </c>
-      <c r="G23" s="7" t="s">
+      <c r="G23" s="6" t="s">
         <v>148</v>
       </c>
-      <c r="H23" s="4" t="s">
+      <c r="H23" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="I23" s="4" t="s">
+      <c r="I23" s="3" t="s">
         <v>149</v>
       </c>
-      <c r="J23" s="4">
+      <c r="J23" s="3">
         <v>22</v>
       </c>
       <c r="K23" s="1" t="s">
@@ -2734,35 +2150,35 @@
         <v>37</v>
       </c>
     </row>
-    <row r="24" ht="43.15" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A24" s="4">
+    <row r="24" spans="1:12" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="3">
         <v>23</v>
       </c>
-      <c r="B24" s="4" t="s">
+      <c r="B24" s="3" t="s">
         <v>151</v>
       </c>
-      <c r="C24" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="D24" s="4" t="s">
+      <c r="C24" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="D24" s="3" t="s">
         <v>152</v>
       </c>
-      <c r="E24" s="7" t="s">
+      <c r="E24" s="6" t="s">
         <v>153</v>
       </c>
-      <c r="F24" s="7" t="s">
+      <c r="F24" s="6" t="s">
         <v>154</v>
       </c>
-      <c r="G24" s="7" t="s">
+      <c r="G24" s="6" t="s">
         <v>155</v>
       </c>
-      <c r="H24" s="4" t="s">
+      <c r="H24" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="I24" s="4" t="s">
+      <c r="I24" s="3" t="s">
         <v>156</v>
       </c>
-      <c r="J24" s="4">
+      <c r="J24" s="3">
         <v>23</v>
       </c>
       <c r="K24" s="1" t="s">
@@ -2772,35 +2188,35 @@
         <v>37</v>
       </c>
     </row>
-    <row r="25" ht="28.9" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A25" s="4">
+    <row r="25" spans="1:12" ht="28.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A25" s="3">
         <v>24</v>
       </c>
-      <c r="B25" s="4" t="s">
+      <c r="B25" s="3" t="s">
         <v>158</v>
       </c>
-      <c r="C25" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="D25" s="4" t="s">
+      <c r="C25" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="D25" s="3" t="s">
         <v>159</v>
       </c>
-      <c r="E25" s="4" t="s">
+      <c r="E25" s="3" t="s">
         <v>160</v>
       </c>
-      <c r="F25" s="4" t="s">
+      <c r="F25" s="3" t="s">
         <v>161</v>
       </c>
-      <c r="G25" s="4" t="s">
+      <c r="G25" s="3" t="s">
         <v>162</v>
       </c>
-      <c r="H25" s="4" t="s">
+      <c r="H25" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="I25" s="4" t="s">
+      <c r="I25" s="3" t="s">
         <v>163</v>
       </c>
-      <c r="J25" s="4">
+      <c r="J25" s="3">
         <v>24</v>
       </c>
       <c r="K25" s="1" t="s">
@@ -2810,35 +2226,35 @@
         <v>165</v>
       </c>
     </row>
-    <row r="26" ht="28.9" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A26" s="4">
+    <row r="26" spans="1:12" ht="28.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A26" s="3">
         <v>25</v>
       </c>
-      <c r="B26" s="4" t="s">
+      <c r="B26" s="3" t="s">
         <v>166</v>
       </c>
-      <c r="C26" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="D26" s="4" t="s">
+      <c r="C26" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="D26" s="3" t="s">
         <v>167</v>
       </c>
-      <c r="E26" s="4" t="s">
+      <c r="E26" s="3" t="s">
         <v>168</v>
       </c>
-      <c r="F26" s="4" t="s">
+      <c r="F26" s="3" t="s">
         <v>161</v>
       </c>
-      <c r="G26" s="4" t="s">
+      <c r="G26" s="3" t="s">
         <v>169</v>
       </c>
-      <c r="H26" s="4" t="s">
+      <c r="H26" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="I26" s="4" t="s">
+      <c r="I26" s="3" t="s">
         <v>170</v>
       </c>
-      <c r="J26" s="4">
+      <c r="J26" s="3">
         <v>25</v>
       </c>
       <c r="K26" s="1" t="s">
@@ -2848,35 +2264,35 @@
         <v>172</v>
       </c>
     </row>
-    <row r="27" ht="43.15" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A27" s="4">
+    <row r="27" spans="1:12" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A27" s="3">
         <v>26</v>
       </c>
-      <c r="B27" s="4" t="s">
+      <c r="B27" s="3" t="s">
         <v>173</v>
       </c>
-      <c r="C27" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="D27" s="4" t="s">
+      <c r="C27" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="D27" s="3" t="s">
         <v>174</v>
       </c>
-      <c r="E27" s="4" t="s">
+      <c r="E27" s="3" t="s">
         <v>175</v>
       </c>
-      <c r="F27" s="4" t="s">
+      <c r="F27" s="3" t="s">
         <v>176</v>
       </c>
-      <c r="G27" s="4" t="s">
+      <c r="G27" s="3" t="s">
         <v>177</v>
       </c>
-      <c r="H27" s="4" t="s">
+      <c r="H27" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="I27" s="4" t="s">
+      <c r="I27" s="3" t="s">
         <v>178</v>
       </c>
-      <c r="J27" s="4">
+      <c r="J27" s="3">
         <v>26</v>
       </c>
       <c r="K27" s="1" t="s">
@@ -2886,35 +2302,35 @@
         <v>37</v>
       </c>
     </row>
-    <row r="28" ht="43.15" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A28" s="4">
+    <row r="28" spans="1:12" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A28" s="3">
         <v>27</v>
       </c>
-      <c r="B28" s="4" t="s">
+      <c r="B28" s="3" t="s">
         <v>180</v>
       </c>
-      <c r="C28" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="D28" s="4" t="s">
+      <c r="C28" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="D28" s="3" t="s">
         <v>181</v>
       </c>
-      <c r="E28" s="4" t="s">
+      <c r="E28" s="3" t="s">
         <v>182</v>
       </c>
-      <c r="F28" s="4" t="s">
+      <c r="F28" s="3" t="s">
         <v>183</v>
       </c>
-      <c r="G28" s="4" t="s">
+      <c r="G28" s="3" t="s">
         <v>184</v>
       </c>
-      <c r="H28" s="4" t="s">
+      <c r="H28" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="I28" s="4" t="s">
+      <c r="I28" s="3" t="s">
         <v>185</v>
       </c>
-      <c r="J28" s="4">
+      <c r="J28" s="3">
         <v>27</v>
       </c>
       <c r="K28" s="1" t="s">
@@ -2924,35 +2340,35 @@
         <v>37</v>
       </c>
     </row>
-    <row r="29" ht="43.15" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A29" s="4">
+    <row r="29" spans="1:12" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A29" s="3">
         <v>28</v>
       </c>
-      <c r="B29" s="4" t="s">
+      <c r="B29" s="3" t="s">
         <v>186</v>
       </c>
-      <c r="C29" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="D29" s="4" t="s">
+      <c r="C29" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="D29" s="3" t="s">
         <v>187</v>
       </c>
-      <c r="E29" s="4" t="s">
+      <c r="E29" s="3" t="s">
         <v>188</v>
       </c>
-      <c r="F29" s="4" t="s">
+      <c r="F29" s="3" t="s">
         <v>189</v>
       </c>
-      <c r="G29" s="4" t="s">
+      <c r="G29" s="3" t="s">
         <v>190</v>
       </c>
-      <c r="H29" s="4" t="s">
+      <c r="H29" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="I29" s="4" t="s">
+      <c r="I29" s="3" t="s">
         <v>191</v>
       </c>
-      <c r="J29" s="4">
+      <c r="J29" s="3">
         <v>28</v>
       </c>
       <c r="K29" s="1" t="s">
@@ -2962,35 +2378,35 @@
         <v>193</v>
       </c>
     </row>
-    <row r="30" ht="43.15" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A30" s="4">
+    <row r="30" spans="1:12" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A30" s="3">
         <v>29</v>
       </c>
-      <c r="B30" s="4" t="s">
+      <c r="B30" s="3" t="s">
         <v>194</v>
       </c>
-      <c r="C30" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="D30" s="4" t="s">
+      <c r="C30" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="D30" s="3" t="s">
         <v>195</v>
       </c>
-      <c r="E30" s="4" t="s">
+      <c r="E30" s="3" t="s">
         <v>196</v>
       </c>
-      <c r="F30" s="4" t="s">
+      <c r="F30" s="3" t="s">
         <v>197</v>
       </c>
-      <c r="G30" s="4" t="s">
+      <c r="G30" s="3" t="s">
         <v>198</v>
       </c>
-      <c r="H30" s="4" t="s">
+      <c r="H30" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="I30" s="4" t="s">
+      <c r="I30" s="3" t="s">
         <v>199</v>
       </c>
-      <c r="J30" s="4">
+      <c r="J30" s="3">
         <v>29</v>
       </c>
       <c r="K30" s="1" t="s">
@@ -3000,73 +2416,73 @@
         <v>37</v>
       </c>
     </row>
-    <row r="31" ht="43.15" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A31" s="4">
+    <row r="31" spans="1:12" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A31" s="3">
         <v>30</v>
       </c>
-      <c r="B31" s="4" t="s">
+      <c r="B31" s="3" t="s">
         <v>201</v>
       </c>
-      <c r="C31" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="D31" s="4" t="s">
+      <c r="C31" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="D31" s="3" t="s">
         <v>202</v>
       </c>
-      <c r="E31" s="4" t="s">
+      <c r="E31" s="3" t="s">
         <v>203</v>
       </c>
-      <c r="F31" s="4" t="s">
+      <c r="F31" s="3" t="s">
         <v>204</v>
       </c>
-      <c r="G31" s="4" t="s">
+      <c r="G31" s="3" t="s">
         <v>205</v>
       </c>
-      <c r="H31" s="4" t="s">
+      <c r="H31" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="I31" s="4" t="s">
+      <c r="I31" s="3" t="s">
         <v>206</v>
       </c>
-      <c r="J31" s="4">
+      <c r="J31" s="3">
         <v>30</v>
       </c>
-      <c r="K31" s="4" t="s">
+      <c r="K31" s="3" t="s">
         <v>207</v>
       </c>
-      <c r="L31" s="4" t="s">
+      <c r="L31" s="3" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="32" ht="43.15" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A32" s="4">
+    <row r="32" spans="1:12" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A32" s="3">
         <v>31</v>
       </c>
-      <c r="B32" s="4" t="s">
+      <c r="B32" s="3" t="s">
         <v>208</v>
       </c>
-      <c r="C32" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="D32" s="4" t="s">
+      <c r="C32" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="D32" s="3" t="s">
         <v>209</v>
       </c>
-      <c r="E32" s="4" t="s">
+      <c r="E32" s="3" t="s">
         <v>210</v>
       </c>
-      <c r="F32" s="4" t="s">
+      <c r="F32" s="3" t="s">
         <v>211</v>
       </c>
-      <c r="G32" s="4" t="s">
+      <c r="G32" s="3" t="s">
         <v>212</v>
       </c>
-      <c r="H32" s="4" t="s">
+      <c r="H32" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="I32" s="4" t="s">
+      <c r="I32" s="3" t="s">
         <v>213</v>
       </c>
-      <c r="J32" s="4">
+      <c r="J32" s="3">
         <v>31</v>
       </c>
       <c r="K32" s="1" t="s">
@@ -3076,35 +2492,35 @@
         <v>193</v>
       </c>
     </row>
-    <row r="33" ht="43.15" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A33" s="4">
+    <row r="33" spans="1:12" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A33" s="3">
         <v>32</v>
       </c>
-      <c r="B33" s="4" t="s">
+      <c r="B33" s="3" t="s">
         <v>215</v>
       </c>
-      <c r="C33" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="D33" s="4" t="s">
+      <c r="C33" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="D33" s="3" t="s">
         <v>216</v>
       </c>
-      <c r="E33" s="4" t="s">
+      <c r="E33" s="3" t="s">
         <v>217</v>
       </c>
-      <c r="F33" s="4" t="s">
+      <c r="F33" s="3" t="s">
         <v>211</v>
       </c>
-      <c r="G33" s="4" t="s">
+      <c r="G33" s="3" t="s">
         <v>212</v>
       </c>
-      <c r="H33" s="4" t="s">
+      <c r="H33" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="I33" s="4" t="s">
+      <c r="I33" s="3" t="s">
         <v>218</v>
       </c>
-      <c r="J33" s="4">
+      <c r="J33" s="3">
         <v>32</v>
       </c>
       <c r="K33" s="1" t="s">
@@ -3114,35 +2530,35 @@
         <v>193</v>
       </c>
     </row>
-    <row r="34" ht="43.15" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A34" s="4">
+    <row r="34" spans="1:12" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A34" s="3">
         <v>33</v>
       </c>
-      <c r="B34" s="4" t="s">
+      <c r="B34" s="3" t="s">
         <v>219</v>
       </c>
-      <c r="C34" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="D34" s="4" t="s">
+      <c r="C34" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="D34" s="3" t="s">
         <v>220</v>
       </c>
-      <c r="E34" s="4" t="s">
+      <c r="E34" s="3" t="s">
         <v>221</v>
       </c>
-      <c r="F34" s="4" t="s">
+      <c r="F34" s="3" t="s">
         <v>222</v>
       </c>
-      <c r="G34" s="4" t="s">
+      <c r="G34" s="3" t="s">
         <v>223</v>
       </c>
-      <c r="H34" s="4" t="s">
+      <c r="H34" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="I34" s="4" t="s">
+      <c r="I34" s="3" t="s">
         <v>224</v>
       </c>
-      <c r="J34" s="4">
+      <c r="J34" s="3">
         <v>33</v>
       </c>
       <c r="K34" s="1" t="s">
@@ -3152,35 +2568,35 @@
         <v>37</v>
       </c>
     </row>
-    <row r="35" ht="43.15" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A35" s="4">
+    <row r="35" spans="1:12" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A35" s="3">
         <v>34</v>
       </c>
-      <c r="B35" s="4" t="s">
+      <c r="B35" s="3" t="s">
         <v>225</v>
       </c>
-      <c r="C35" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="D35" s="4" t="s">
+      <c r="C35" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="D35" s="3" t="s">
         <v>226</v>
       </c>
-      <c r="E35" s="4" t="s">
+      <c r="E35" s="3" t="s">
         <v>227</v>
       </c>
-      <c r="F35" s="4" t="s">
+      <c r="F35" s="3" t="s">
         <v>228</v>
       </c>
-      <c r="G35" s="4" t="s">
+      <c r="G35" s="3" t="s">
         <v>229</v>
       </c>
-      <c r="H35" s="4" t="s">
+      <c r="H35" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="I35" s="4" t="s">
+      <c r="I35" s="3" t="s">
         <v>230</v>
       </c>
-      <c r="J35" s="4">
+      <c r="J35" s="3">
         <v>34</v>
       </c>
       <c r="K35" s="1" t="s">
@@ -3190,35 +2606,35 @@
         <v>37</v>
       </c>
     </row>
-    <row r="36" ht="43.15" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A36" s="4">
+    <row r="36" spans="1:12" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A36" s="3">
         <v>35</v>
       </c>
-      <c r="B36" s="4" t="s">
+      <c r="B36" s="3" t="s">
         <v>231</v>
       </c>
-      <c r="C36" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="D36" s="4" t="s">
+      <c r="C36" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="D36" s="3" t="s">
         <v>232</v>
       </c>
-      <c r="E36" s="4" t="s">
+      <c r="E36" s="3" t="s">
         <v>233</v>
       </c>
-      <c r="F36" s="4" t="s">
+      <c r="F36" s="3" t="s">
         <v>234</v>
       </c>
-      <c r="G36" s="4" t="s">
+      <c r="G36" s="3" t="s">
         <v>235</v>
       </c>
-      <c r="H36" s="4" t="s">
+      <c r="H36" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="I36" s="4" t="s">
+      <c r="I36" s="3" t="s">
         <v>236</v>
       </c>
-      <c r="J36" s="4">
+      <c r="J36" s="3">
         <v>35</v>
       </c>
       <c r="K36" s="1" t="s">
@@ -3228,35 +2644,35 @@
         <v>37</v>
       </c>
     </row>
-    <row r="37" ht="43.15" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A37" s="4">
+    <row r="37" spans="1:12" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A37" s="3">
         <v>36</v>
       </c>
-      <c r="B37" s="4" t="s">
+      <c r="B37" s="3" t="s">
         <v>237</v>
       </c>
-      <c r="C37" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="D37" s="4" t="s">
+      <c r="C37" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="D37" s="3" t="s">
         <v>238</v>
       </c>
-      <c r="E37" s="4" t="s">
+      <c r="E37" s="3" t="s">
         <v>233</v>
       </c>
-      <c r="F37" s="4" t="s">
+      <c r="F37" s="3" t="s">
         <v>239</v>
       </c>
-      <c r="G37" s="4" t="s">
+      <c r="G37" s="3" t="s">
         <v>240</v>
       </c>
-      <c r="H37" s="4" t="s">
+      <c r="H37" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="I37" s="4" t="s">
+      <c r="I37" s="3" t="s">
         <v>241</v>
       </c>
-      <c r="J37" s="4">
+      <c r="J37" s="3">
         <v>36</v>
       </c>
       <c r="K37" s="1" t="s">
@@ -3266,35 +2682,35 @@
         <v>37</v>
       </c>
     </row>
-    <row r="38" ht="28.9" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A38" s="4">
+    <row r="38" spans="1:12" ht="28.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A38" s="3">
         <v>37</v>
       </c>
-      <c r="B38" s="4" t="s">
+      <c r="B38" s="3" t="s">
         <v>242</v>
       </c>
-      <c r="C38" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="D38" s="4" t="s">
+      <c r="C38" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="D38" s="3" t="s">
         <v>243</v>
       </c>
-      <c r="E38" s="4" t="s">
+      <c r="E38" s="3" t="s">
         <v>244</v>
       </c>
-      <c r="F38" s="4" t="s">
+      <c r="F38" s="3" t="s">
         <v>245</v>
       </c>
-      <c r="G38" s="4" t="s">
+      <c r="G38" s="3" t="s">
         <v>246</v>
       </c>
-      <c r="H38" s="4" t="s">
+      <c r="H38" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="I38" s="4" t="s">
+      <c r="I38" s="3" t="s">
         <v>247</v>
       </c>
-      <c r="J38" s="4">
+      <c r="J38" s="3">
         <v>37</v>
       </c>
       <c r="K38" s="1" t="s">
@@ -3305,130 +2721,452 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L38"/>
+  <autoFilter ref="A1:L38" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{608A33FA-BF70-47B7-A2EC-5C01069E6791}">
+  <dimension ref="A1:C38"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="3.5546875" style="1" customWidth="1"/>
+    <col min="2" max="2" width="7.44140625" style="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" s="3">
+        <v>1</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" s="3">
+        <v>2</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" s="3">
+        <v>3</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" s="3">
+        <v>4</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" s="3">
+        <v>5</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7" s="3">
+        <v>6</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A8" s="3">
+        <v>7</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A9" s="3">
+        <v>8</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A10" s="3">
+        <v>9</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A11" s="3">
+        <v>10</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A12" s="3">
+        <v>11</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A13" s="3">
+        <v>12</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A14" s="3">
+        <v>13</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A15" s="3">
+        <v>14</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A16" s="3">
+        <v>15</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A17" s="3">
+        <v>16</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A18" s="3">
+        <v>17</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A19" s="3">
+        <v>18</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A20" s="3">
+        <v>19</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A21" s="3">
+        <v>20</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A22" s="3">
+        <v>21</v>
+      </c>
+      <c r="B22" s="3" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A23" s="3">
+        <v>22</v>
+      </c>
+      <c r="B23" s="3" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A24" s="3">
+        <v>23</v>
+      </c>
+      <c r="B24" s="3" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A25" s="3">
+        <v>24</v>
+      </c>
+      <c r="B25" s="3" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A26" s="3">
+        <v>25</v>
+      </c>
+      <c r="B26" s="3" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A27" s="3">
+        <v>26</v>
+      </c>
+      <c r="B27" s="3" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A28" s="3">
+        <v>27</v>
+      </c>
+      <c r="B28" s="3" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A29" s="3">
+        <v>28</v>
+      </c>
+      <c r="B29" s="3" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A30" s="3">
+        <v>29</v>
+      </c>
+      <c r="B30" s="3" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A31" s="3">
+        <v>30</v>
+      </c>
+      <c r="B31" s="3" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A32" s="3">
+        <v>31</v>
+      </c>
+      <c r="B32" s="3" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A33" s="3">
+        <v>32</v>
+      </c>
+      <c r="B33" s="3" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A34" s="3">
+        <v>33</v>
+      </c>
+      <c r="B34" s="3" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A35" s="3">
+        <v>34</v>
+      </c>
+      <c r="B35" s="3" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A36" s="3">
+        <v>35</v>
+      </c>
+      <c r="B36" s="3" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A37" s="3">
+        <v>36</v>
+      </c>
+      <c r="B37" s="3" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A38" s="3">
+        <v>37</v>
+      </c>
+      <c r="B38" s="3" t="s">
+        <v>242</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <sheetPr>
     <tabColor rgb="FFFFFF00"/>
   </sheetPr>
   <dimension ref="A1:D8"/>
-  <sheetFormatPr defaultRowHeight="14.45" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="13.28515625" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="13.33203125" defaultRowHeight="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="5.28515625" style="16" customWidth="1"/>
-    <col min="2" max="2" width="26.28515625" style="16" customWidth="1"/>
-    <col min="3" max="3" width="90.28515625" style="16" customWidth="1"/>
-    <col min="4" max="4" width="45" style="16" customWidth="1"/>
-    <col min="5" max="16384" width="13.28515625" style="16" customWidth="1"/>
+    <col min="1" max="1" width="5.33203125" style="10" customWidth="1"/>
+    <col min="2" max="2" width="26.33203125" style="10" customWidth="1"/>
+    <col min="3" max="3" width="90.33203125" style="10" customWidth="1"/>
+    <col min="4" max="4" width="45" style="10" customWidth="1"/>
+    <col min="5" max="5" width="13.33203125" style="10" customWidth="1"/>
+    <col min="6" max="16384" width="13.33203125" style="10"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" s="17" t="s">
-        <v>274</v>
-      </c>
-      <c r="B1" s="17"/>
-      <c r="C1" s="17"/>
-      <c r="D1" s="17"/>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" s="18" t="s">
-        <v>275</v>
-      </c>
-      <c r="B2" s="18" t="s">
-        <v>276</v>
-      </c>
-      <c r="C2" s="18" t="s">
-        <v>277</v>
-      </c>
-      <c r="D2" s="18" t="s">
-        <v>278</v>
-      </c>
-    </row>
-    <row r="3" ht="28.9" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" s="19">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A1" s="13" t="s">
+        <v>248</v>
+      </c>
+      <c r="B1" s="13"/>
+      <c r="C1" s="13"/>
+      <c r="D1" s="13"/>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A2" s="11" t="s">
+        <v>249</v>
+      </c>
+      <c r="B2" s="11" t="s">
+        <v>250</v>
+      </c>
+      <c r="C2" s="11" t="s">
+        <v>251</v>
+      </c>
+      <c r="D2" s="11" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="28.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="12">
         <v>1</v>
       </c>
-      <c r="B3" s="19" t="s">
-        <v>279</v>
-      </c>
-      <c r="C3" s="19" t="s">
-        <v>280</v>
-      </c>
-      <c r="D3" s="19" t="s">
-        <v>281</v>
-      </c>
-    </row>
-    <row r="4" ht="28.9" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" s="19">
+      <c r="B3" s="12" t="s">
+        <v>253</v>
+      </c>
+      <c r="C3" s="12" t="s">
+        <v>254</v>
+      </c>
+      <c r="D3" s="12" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="28.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="12">
         <v>2</v>
       </c>
-      <c r="B4" s="19" t="s">
-        <v>282</v>
-      </c>
-      <c r="C4" s="19" t="s">
-        <v>283</v>
-      </c>
-      <c r="D4" s="19" t="s">
-        <v>284</v>
-      </c>
-    </row>
-    <row r="5" ht="28.9" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" s="19">
+      <c r="B4" s="12" t="s">
+        <v>256</v>
+      </c>
+      <c r="C4" s="12" t="s">
+        <v>257</v>
+      </c>
+      <c r="D4" s="12" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="28.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="12">
         <v>3</v>
       </c>
-      <c r="B5" s="19" t="s">
-        <v>285</v>
-      </c>
-      <c r="C5" s="19" t="s">
+      <c r="B5" s="12" t="s">
+        <v>259</v>
+      </c>
+      <c r="C5" s="12" t="s">
         <v>184</v>
       </c>
-      <c r="D5" s="19" t="s">
-        <v>284</v>
-      </c>
-    </row>
-    <row r="6" ht="43.15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A6" s="19">
+      <c r="D5" s="12" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="12">
         <v>4</v>
       </c>
-      <c r="B6" s="19" t="s">
-        <v>286</v>
-      </c>
-      <c r="C6" s="19" t="s">
-        <v>287</v>
-      </c>
-      <c r="D6" s="19" t="s">
-        <v>284</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7" s="19">
+      <c r="B6" s="12" t="s">
+        <v>260</v>
+      </c>
+      <c r="C6" s="12" t="s">
+        <v>261</v>
+      </c>
+      <c r="D6" s="12" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A7" s="12">
         <v>5</v>
       </c>
-      <c r="B7" s="19" t="s">
-        <v>288</v>
-      </c>
-      <c r="C7" s="19" t="s">
-        <v>289</v>
-      </c>
-      <c r="D7" s="19" t="s">
-        <v>281</v>
-      </c>
-    </row>
-    <row r="8" ht="28.9" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A8" s="19">
+      <c r="B7" s="12" t="s">
+        <v>262</v>
+      </c>
+      <c r="C7" s="12" t="s">
+        <v>263</v>
+      </c>
+      <c r="D7" s="12" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="28.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="12">
         <v>6</v>
       </c>
-      <c r="B8" s="19" t="s">
-        <v>290</v>
-      </c>
-      <c r="C8" s="19" t="s">
-        <v>291</v>
-      </c>
-      <c r="D8" s="19" t="s">
-        <v>284</v>
+      <c r="B8" s="12" t="s">
+        <v>264</v>
+      </c>
+      <c r="C8" s="12" t="s">
+        <v>265</v>
+      </c>
+      <c r="D8" s="12" t="s">
+        <v>258</v>
       </c>
     </row>
   </sheetData>
@@ -3437,153 +3175,4 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <sheetPr>
-    <tabColor rgb="FFFFFF00"/>
-  </sheetPr>
-  <dimension ref="B1:B291"/>
-  <sheetFormatPr defaultRowHeight="14.45" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="9.28515625" customHeight="1"/>
-  <cols>
-    <col min="1" max="1" width="2" style="11" customWidth="1"/>
-    <col min="2" max="2" width="120" style="11" customWidth="1"/>
-    <col min="3" max="16384" width="9.28515625" style="11" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="32.25" customHeight="1" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B1" s="12" t="s">
-        <v>248</v>
-      </c>
-    </row>
-    <row r="3" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B3" s="13" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="4" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B4" s="14" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="27" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B27" s="13" t="s">
-        <v>251</v>
-      </c>
-    </row>
-    <row r="28" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B28" s="14" t="s">
-        <v>252</v>
-      </c>
-    </row>
-    <row r="51" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B51" s="13" t="s">
-        <v>253</v>
-      </c>
-    </row>
-    <row r="52" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B52" s="14" t="s">
-        <v>254</v>
-      </c>
-    </row>
-    <row r="75" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B75" s="13" t="s">
-        <v>255</v>
-      </c>
-    </row>
-    <row r="76" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B76" s="14" t="s">
-        <v>256</v>
-      </c>
-    </row>
-    <row r="99" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B99" s="13" t="s">
-        <v>257</v>
-      </c>
-    </row>
-    <row r="100" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B100" s="14" t="s">
-        <v>258</v>
-      </c>
-    </row>
-    <row r="123" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B123" s="13" t="s">
-        <v>259</v>
-      </c>
-    </row>
-    <row r="124" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B124" s="14" t="s">
-        <v>260</v>
-      </c>
-    </row>
-    <row r="147" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B147" s="13" t="s">
-        <v>261</v>
-      </c>
-    </row>
-    <row r="148" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B148" s="14" t="s">
-        <v>262</v>
-      </c>
-    </row>
-    <row r="171" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B171" s="13" t="s">
-        <v>263</v>
-      </c>
-    </row>
-    <row r="172" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B172" s="14" t="s">
-        <v>264</v>
-      </c>
-    </row>
-    <row r="195" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B195" s="13" t="s">
-        <v>265</v>
-      </c>
-    </row>
-    <row r="196" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B196" s="14" t="s">
-        <v>266</v>
-      </c>
-    </row>
-    <row r="219" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B219" s="13" t="s">
-        <v>267</v>
-      </c>
-    </row>
-    <row r="220" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B220" s="14" t="s">
-        <v>268</v>
-      </c>
-    </row>
-    <row r="243" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B243" s="13" t="s">
-        <v>269</v>
-      </c>
-    </row>
-    <row r="244" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B244" s="14" t="s">
-        <v>270</v>
-      </c>
-    </row>
-    <row r="267" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B267" s="13" t="s">
-        <v>271</v>
-      </c>
-    </row>
-    <row r="268" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B268" s="14" t="s">
-        <v>272</v>
-      </c>
-    </row>
-    <row r="291" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B291" s="15" t="s">
-        <v>273</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
-</worksheet>
 </file>
</xml_diff>